<commit_message>
feat(F-NAR-016): TREE-DIF-046 passe agent après apply
</commit_message>
<xml_diff>
--- a/stories/arbres/TREE-DIF-046.xlsx
+++ b/stories/arbres/TREE-DIF-046.xlsx
@@ -2307,12 +2307,12 @@
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>Le panier arrive près de l'étal de papier. Le panier bute contre une caisse de papier. Des moulinets pendent, tous mêlés. C'est ici ? C'est le rouge, près du. Le mot s'arrête au milieu. Près du quoi ? Victorino referme sa bouche, tout net. Ils se ressemblent tous, là-haut. On fait comment, Victorino ?</t>
+          <t>Le panier arrive près de l'étal de papier. Il bute contre une caisse de papier. Des moulinets pendent, tous mêlés. C'est ici ? C'est le rouge, près du. Le mot s'arrête au milieu. Près du quoi ? Victorino referme sa bouche, tout net. Ils se ressemblent tous, là-haut. On fait comment, Victorino ?</t>
         </is>
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>Le panier arrive près de l'étal de papier. Le panier bute contre une caisse de papier. Des moulinets pendent, tous mêlés. C'est ici ? C'est le rouge, près du. Le mot s'arrête au milieu. Près du quoi ? Victorino referme sa bouche, tout net. Ils se ressemblent tous, là-haut. On fait comment, Victorino ?</t>
+          <t>Le panier arrive près de l'étal de papier. Il bute contre une caisse de papier. Des moulinets pendent, tous mêlés. C'est ici ? C'est le rouge, près du. Le mot s'arrête au milieu. Près du quoi ? Victorino referme sa bouche, tout net. Ils se ressemblent tous, là-haut. On fait comment, Victorino ?</t>
         </is>
       </c>
       <c r="G8" s="2" t="inlineStr">
@@ -2448,7 +2448,7 @@
       <c r="AW8" t="inlineStr">
         <is>
           <t>narrateur|Le panier arrive près de l'étal de papier.
-narrateur|Le panier bute contre une caisse de papier.
+narrateur|Il bute contre une caisse de papier.
 narrateur|Des moulinets pendent, tous mêlés.
 enfant-m|C'est ici ?
 papa|C'est le rouge, près du.
@@ -3726,12 +3726,12 @@
       </c>
       <c r="E16" s="2" t="inlineStr">
         <is>
-          <t>Le panier arrive près de la fontaine. Le panier se mouille un peu, au bord. Il est là-dedans, le rouge ? Il est près de l'. L'eau couvre le mot, tout fort. Des gouttes tapent le bord, déjà. Près de l'eau ? Victorino recule d'un pas, puis attend. On n'entend plus la fin. Tu trouves comment ?</t>
+          <t>Le panier arrive près de la fontaine. Il se mouille un peu, au bord. Il est là, le rouge ? Il est près de l'. L'eau couvre le mot, tout fort. Des gouttes tapent le bord, déjà. Près de l'eau ? Victorino recule d'un pas, puis attend. On n'entend plus la fin. Tu trouves comment ?</t>
         </is>
       </c>
       <c r="F16" s="2" t="inlineStr">
         <is>
-          <t>Le panier arrive près de la fontaine. Le panier se mouille un peu, au bord. Il est là-dedans, le rouge ? Il est près de l'. L'eau couvre le mot, tout fort. Des gouttes tapent le bord, déjà. Près de l'eau ? Victorino recule d'un pas, puis attend. On n'entend plus la fin. Tu trouves comment ?</t>
+          <t>Le panier arrive près de la fontaine. Il se mouille un peu, au bord. Il est là, le rouge ? Il est près de l'. L'eau couvre le mot, tout fort. Des gouttes tapent le bord, déjà. Près de l'eau ? Victorino recule d'un pas, puis attend. On n'entend plus la fin. Tu trouves comment ?</t>
         </is>
       </c>
       <c r="G16" s="2" t="inlineStr">
@@ -3867,8 +3867,8 @@
       <c r="AW16" t="inlineStr">
         <is>
           <t>narrateur|Le panier arrive près de la fontaine.
-narrateur|Le panier se mouille un peu, au bord.
-enfant-m|Il est là-dedans, le rouge ?
+narrateur|Il se mouille un peu, au bord.
+enfant-m|Il est là, le rouge ?
 maman|Il est près de l'.
 narrateur|L'eau couvre le mot, tout fort.
 narrateur|Des gouttes tapent le bord, déjà.
@@ -4273,12 +4273,12 @@
       </c>
       <c r="E19" s="2" t="inlineStr">
         <is>
-          <t>Loin de l'eau, le rouge était là. Tu as fini, papa. Oui, le mot était long. Merci d'avoir reculé sans crier. Le panier tient le bâton, tout droit. Une goutte sèche déjà sur le bâton. Victorino fait tourner le rouge, tout près. La fontaine redevient une fontaine, tout simple.</t>
+          <t>Loin de l'eau, le rouge était là. Tu as fini, papa. Oui, le mot était long. Tu as reculé, tout doux. Le panier tient le bâton, tout droit. Une goutte sèche déjà sur le bâton. Victorino fait tourner le rouge, tout près. La fontaine redevient une fontaine, tout simple.</t>
         </is>
       </c>
       <c r="F19" s="2" t="inlineStr">
         <is>
-          <t>Loin de l'eau, le rouge était là. Tu as fini, papa. Oui, le mot était long. Merci d'avoir reculé sans crier. Le panier tient le bâton, tout droit. Une goutte sèche déjà sur le bâton. Victorino fait tourner le rouge, tout près. La fontaine redevient une fontaine, tout simple.</t>
+          <t>Loin de l'eau, le rouge était là. Tu as fini, papa. Oui, le mot était long. Tu as reculé, tout doux. Le panier tient le bâton, tout droit. Une goutte sèche déjà sur le bâton. Victorino fait tourner le rouge, tout près. La fontaine redevient une fontaine, tout simple.</t>
         </is>
       </c>
       <c r="G19" s="2" t="inlineStr">
@@ -4416,7 +4416,7 @@
           <t>narrateur|Loin de l'eau, le rouge était là.
 enfant-m|Tu as fini, papa.
 papa|Oui, le mot était long.
-maman|Merci d'avoir reculé sans crier.
+maman|Tu as reculé, tout doux.
 narrateur|Le panier tient le bâton, tout droit.
 narrateur|Une goutte sèche déjà sur le bâton.
 narrateur|Victorino fait tourner le rouge, tout près.
@@ -5145,12 +5145,12 @@
       </c>
       <c r="E24" s="2" t="inlineStr">
         <is>
-          <t>Le panier arrive sous l'auvent bleu. Le panier lève le nez, trop bas encore. Tout en haut ? Tout en haut, près du. Papa s'arrête, les lèvres encore rondes. Près du bord ? Victorino garde sa bouche fermée, après. Le haut est trop loin, pour lui. Un tabouret dort près du mur. Tu fais quoi, alors ?</t>
+          <t>Le panier arrive sous l'auvent bleu. Il reste trop bas, encore. Tout en haut ? Tout en haut, près du. Papa s'arrête, les lèvres encore rondes. Près du bord ? Victorino garde sa bouche fermée, après. Le haut est trop loin, pour lui. Un tabouret dort près du mur. Tu fais quoi, alors ?</t>
         </is>
       </c>
       <c r="F24" s="2" t="inlineStr">
         <is>
-          <t>Le panier arrive sous l'auvent bleu. Le panier lève le nez, trop bas encore. Tout en haut ? Tout en haut, près du. Papa s'arrête, les lèvres encore rondes. Près du bord ? Victorino garde sa bouche fermée, après. Le haut est trop loin, pour lui. Un tabouret dort près du mur. Tu fais quoi, alors ?</t>
+          <t>Le panier arrive sous l'auvent bleu. Il reste trop bas, encore. Tout en haut ? Tout en haut, près du. Papa s'arrête, les lèvres encore rondes. Près du bord ? Victorino garde sa bouche fermée, après. Le haut est trop loin, pour lui. Un tabouret dort près du mur. Tu fais quoi, alors ?</t>
         </is>
       </c>
       <c r="G24" s="2" t="inlineStr">
@@ -5286,7 +5286,7 @@
       <c r="AW24" t="inlineStr">
         <is>
           <t>narrateur|Le panier arrive sous l'auvent bleu.
-narrateur|Le panier lève le nez, trop bas encore.
+narrateur|Il reste trop bas, encore.
 enfant-m|Tout en haut ?
 papa|Tout en haut, près du.
 narrateur|Papa s'arrête, les lèvres encore rondes.
@@ -7300,12 +7300,12 @@
       </c>
       <c r="E36" s="2" t="inlineStr">
         <is>
-          <t>La ficelle arrive près de l'étal de papier. La ficelle s'accroche à un clou, déjà. Des moulinets pendent, tous mêlés. C'est ici ? C'est le rouge, près du. Le mot s'arrête au milieu. Près du quoi ? Victorino referme sa bouche, tout net. Ils se ressemblent tous, là-haut. On fait comment, Victorino ?</t>
+          <t>La ficelle arrive près de l'étal de papier. Elle s'accroche à un clou, déjà. Des moulinets pendent, tous mêlés. C'est ici ? C'est le rouge, près du. Le mot s'arrête au milieu. Près du quoi ? Victorino referme sa bouche, tout net. Ils se ressemblent tous, là-haut. On fait comment, Victorino ?</t>
         </is>
       </c>
       <c r="F36" s="2" t="inlineStr">
         <is>
-          <t>La ficelle arrive près de l'étal de papier. La ficelle s'accroche à un clou, déjà. Des moulinets pendent, tous mêlés. C'est ici ? C'est le rouge, près du. Le mot s'arrête au milieu. Près du quoi ? Victorino referme sa bouche, tout net. Ils se ressemblent tous, là-haut. On fait comment, Victorino ?</t>
+          <t>La ficelle arrive près de l'étal de papier. Elle s'accroche à un clou, déjà. Des moulinets pendent, tous mêlés. C'est ici ? C'est le rouge, près du. Le mot s'arrête au milieu. Près du quoi ? Victorino referme sa bouche, tout net. Ils se ressemblent tous, là-haut. On fait comment, Victorino ?</t>
         </is>
       </c>
       <c r="G36" s="2" t="inlineStr">
@@ -7441,7 +7441,7 @@
       <c r="AW36" t="inlineStr">
         <is>
           <t>narrateur|La ficelle arrive près de l'étal de papier.
-narrateur|La ficelle s'accroche à un clou, déjà.
+narrateur|Elle s'accroche à un clou, déjà.
 narrateur|Des moulinets pendent, tous mêlés.
 enfant-m|C'est ici ?
 papa|C'est le rouge, près du.
@@ -8719,12 +8719,12 @@
       </c>
       <c r="E44" s="2" t="inlineStr">
         <is>
-          <t>La ficelle arrive près de la fontaine. La ficelle boit une goutte, tout net. Il est là-dedans, le rouge ? Il est près de l'. L'eau couvre le mot, tout fort. Des gouttes tapent le bord, déjà. Près de l'eau ? Victorino recule d'un pas, puis attend. On n'entend plus la fin. Tu trouves comment ?</t>
+          <t>La ficelle arrive près de la fontaine. Elle boit une goutte, tout net. Il est là, le rouge ? Il est près de l'. L'eau couvre le mot, tout fort. Des gouttes tapent le bord, déjà. Près de l'eau ? Victorino recule d'un pas, puis attend. On n'entend plus la fin. Tu trouves comment ?</t>
         </is>
       </c>
       <c r="F44" s="2" t="inlineStr">
         <is>
-          <t>La ficelle arrive près de la fontaine. La ficelle boit une goutte, tout net. Il est là-dedans, le rouge ? Il est près de l'. L'eau couvre le mot, tout fort. Des gouttes tapent le bord, déjà. Près de l'eau ? Victorino recule d'un pas, puis attend. On n'entend plus la fin. Tu trouves comment ?</t>
+          <t>La ficelle arrive près de la fontaine. Elle boit une goutte, tout net. Il est là, le rouge ? Il est près de l'. L'eau couvre le mot, tout fort. Des gouttes tapent le bord, déjà. Près de l'eau ? Victorino recule d'un pas, puis attend. On n'entend plus la fin. Tu trouves comment ?</t>
         </is>
       </c>
       <c r="G44" s="2" t="inlineStr">
@@ -8860,8 +8860,8 @@
       <c r="AW44" t="inlineStr">
         <is>
           <t>narrateur|La ficelle arrive près de la fontaine.
-narrateur|La ficelle boit une goutte, tout net.
-enfant-m|Il est là-dedans, le rouge ?
+narrateur|Elle boit une goutte, tout net.
+enfant-m|Il est là, le rouge ?
 maman|Il est près de l'.
 narrateur|L'eau couvre le mot, tout fort.
 narrateur|Des gouttes tapent le bord, déjà.
@@ -9266,12 +9266,12 @@
       </c>
       <c r="E47" s="2" t="inlineStr">
         <is>
-          <t>Loin de l'eau, le rouge était là. Tu as fini, papa. Oui, le mot était long. Merci d'avoir reculé sans crier. La ficelle serre le bois, tout net. Une goutte sèche déjà sur le bâton. Victorino fait tourner le rouge, tout près. La fontaine redevient une fontaine, tout simple.</t>
+          <t>Loin de l'eau, le rouge était là. Tu as fini, papa. Oui, le mot était long. Tu as reculé, tout doux. La ficelle serre le bois, tout net. Une goutte sèche déjà sur le bâton. Victorino fait tourner le rouge, tout près. La fontaine redevient une fontaine, tout simple.</t>
         </is>
       </c>
       <c r="F47" s="2" t="inlineStr">
         <is>
-          <t>Loin de l'eau, le rouge était là. Tu as fini, papa. Oui, le mot était long. Merci d'avoir reculé sans crier. La ficelle serre le bois, tout net. Une goutte sèche déjà sur le bâton. Victorino fait tourner le rouge, tout près. La fontaine redevient une fontaine, tout simple.</t>
+          <t>Loin de l'eau, le rouge était là. Tu as fini, papa. Oui, le mot était long. Tu as reculé, tout doux. La ficelle serre le bois, tout net. Une goutte sèche déjà sur le bâton. Victorino fait tourner le rouge, tout près. La fontaine redevient une fontaine, tout simple.</t>
         </is>
       </c>
       <c r="G47" s="2" t="inlineStr">
@@ -9409,7 +9409,7 @@
           <t>narrateur|Loin de l'eau, le rouge était là.
 enfant-m|Tu as fini, papa.
 papa|Oui, le mot était long.
-maman|Merci d'avoir reculé sans crier.
+maman|Tu as reculé, tout doux.
 narrateur|La ficelle serre le bois, tout net.
 narrateur|Une goutte sèche déjà sur le bâton.
 narrateur|Victorino fait tourner le rouge, tout près.
@@ -10138,12 +10138,12 @@
       </c>
       <c r="E52" s="2" t="inlineStr">
         <is>
-          <t>La ficelle arrive sous l'auvent bleu. La ficelle pend, trop courte, sous le bleu. Tout en haut ? Tout en haut, près du. Papa s'arrête, les lèvres encore rondes. Près du bord ? Victorino garde sa bouche fermée, après. Le haut est trop loin, pour lui. Un tabouret dort près du mur. Tu fais quoi, alors ?</t>
+          <t>La ficelle arrive sous l'auvent bleu. Elle pend, trop courte, sous le bleu. Tout en haut ? Tout en haut, près du. Papa s'arrête, les lèvres encore rondes. Près du bord ? Victorino garde sa bouche fermée, après. Le haut est trop loin, pour lui. Un tabouret dort près du mur. Tu fais quoi, alors ?</t>
         </is>
       </c>
       <c r="F52" s="2" t="inlineStr">
         <is>
-          <t>La ficelle arrive sous l'auvent bleu. La ficelle pend, trop courte, sous le bleu. Tout en haut ? Tout en haut, près du. Papa s'arrête, les lèvres encore rondes. Près du bord ? Victorino garde sa bouche fermée, après. Le haut est trop loin, pour lui. Un tabouret dort près du mur. Tu fais quoi, alors ?</t>
+          <t>La ficelle arrive sous l'auvent bleu. Elle pend, trop courte, sous le bleu. Tout en haut ? Tout en haut, près du. Papa s'arrête, les lèvres encore rondes. Près du bord ? Victorino garde sa bouche fermée, après. Le haut est trop loin, pour lui. Un tabouret dort près du mur. Tu fais quoi, alors ?</t>
         </is>
       </c>
       <c r="G52" s="2" t="inlineStr">
@@ -10279,7 +10279,7 @@
       <c r="AW52" t="inlineStr">
         <is>
           <t>narrateur|La ficelle arrive sous l'auvent bleu.
-narrateur|La ficelle pend, trop courte, sous le bleu.
+narrateur|Elle pend, trop courte, sous le bleu.
 enfant-m|Tout en haut ?
 papa|Tout en haut, près du.
 narrateur|Papa s'arrête, les lèvres encore rondes.
@@ -12293,12 +12293,12 @@
       </c>
       <c r="E64" s="2" t="inlineStr">
         <is>
-          <t>La bourse arrive près de l'étal de papier. La bourse tape le bois, un petit toc. Des moulinets pendent, tous mêlés. C'est ici ? C'est le rouge, près du. Le mot s'arrête au milieu. Près du quoi ? Victorino referme sa bouche, tout net. Ils se ressemblent tous, là-haut. On fait comment, Victorino ?</t>
+          <t>La bourse arrive près de l'étal de papier. Elle tape le bois, un petit toc. Des moulinets pendent, tous mêlés. C'est ici ? C'est le rouge, près du. Le mot s'arrête au milieu. Près du quoi ? Victorino referme sa bouche, tout net. Ils se ressemblent tous, là-haut. On fait comment, Victorino ?</t>
         </is>
       </c>
       <c r="F64" s="2" t="inlineStr">
         <is>
-          <t>La bourse arrive près de l'étal de papier. La bourse tape le bois, un petit toc. Des moulinets pendent, tous mêlés. C'est ici ? C'est le rouge, près du. Le mot s'arrête au milieu. Près du quoi ? Victorino referme sa bouche, tout net. Ils se ressemblent tous, là-haut. On fait comment, Victorino ?</t>
+          <t>La bourse arrive près de l'étal de papier. Elle tape le bois, un petit toc. Des moulinets pendent, tous mêlés. C'est ici ? C'est le rouge, près du. Le mot s'arrête au milieu. Près du quoi ? Victorino referme sa bouche, tout net. Ils se ressemblent tous, là-haut. On fait comment, Victorino ?</t>
         </is>
       </c>
       <c r="G64" s="2" t="inlineStr">
@@ -12434,7 +12434,7 @@
       <c r="AW64" t="inlineStr">
         <is>
           <t>narrateur|La bourse arrive près de l'étal de papier.
-narrateur|La bourse tape le bois, un petit toc.
+narrateur|Elle tape le bois, un petit toc.
 narrateur|Des moulinets pendent, tous mêlés.
 enfant-m|C'est ici ?
 papa|C'est le rouge, près du.
@@ -13712,12 +13712,12 @@
       </c>
       <c r="E72" s="2" t="inlineStr">
         <is>
-          <t>La bourse arrive près de la fontaine. La bourse cliquette sous l'eau qui vole. Il est là-dedans, le rouge ? Il est près de l'. L'eau couvre le mot, tout fort. Des gouttes tapent le bord, déjà. Près de l'eau ? Victorino recule d'un pas, puis attend. On n'entend plus la fin. Tu trouves comment ?</t>
+          <t>La bourse arrive près de la fontaine. Elle cliquette sous l'eau qui vole. Il est là, le rouge ? Il est près de l'. L'eau couvre le mot, tout fort. Des gouttes tapent le bord, déjà. Près de l'eau ? Victorino recule d'un pas, puis attend. On n'entend plus la fin. Tu trouves comment ?</t>
         </is>
       </c>
       <c r="F72" s="2" t="inlineStr">
         <is>
-          <t>La bourse arrive près de la fontaine. La bourse cliquette sous l'eau qui vole. Il est là-dedans, le rouge ? Il est près de l'. L'eau couvre le mot, tout fort. Des gouttes tapent le bord, déjà. Près de l'eau ? Victorino recule d'un pas, puis attend. On n'entend plus la fin. Tu trouves comment ?</t>
+          <t>La bourse arrive près de la fontaine. Elle cliquette sous l'eau qui vole. Il est là, le rouge ? Il est près de l'. L'eau couvre le mot, tout fort. Des gouttes tapent le bord, déjà. Près de l'eau ? Victorino recule d'un pas, puis attend. On n'entend plus la fin. Tu trouves comment ?</t>
         </is>
       </c>
       <c r="G72" s="2" t="inlineStr">
@@ -13853,8 +13853,8 @@
       <c r="AW72" t="inlineStr">
         <is>
           <t>narrateur|La bourse arrive près de la fontaine.
-narrateur|La bourse cliquette sous l'eau qui vole.
-enfant-m|Il est là-dedans, le rouge ?
+narrateur|Elle cliquette sous l'eau qui vole.
+enfant-m|Il est là, le rouge ?
 maman|Il est près de l'.
 narrateur|L'eau couvre le mot, tout fort.
 narrateur|Des gouttes tapent le bord, déjà.
@@ -14259,12 +14259,12 @@
       </c>
       <c r="E75" s="2" t="inlineStr">
         <is>
-          <t>Loin de l'eau, le rouge était là. Tu as fini, papa. Oui, le mot était long. Merci d'avoir reculé sans crier. La bourse cliquette une fois, puis se tait. Une goutte sèche déjà sur le bâton. Victorino fait tourner le rouge, tout près. La fontaine redevient une fontaine, tout simple.</t>
+          <t>Loin de l'eau, le rouge était là. Tu as fini, papa. Oui, le mot était long. Tu as reculé, tout doux. La bourse cliquette une fois, puis se tait. Une goutte sèche déjà sur le bâton. Victorino fait tourner le rouge, tout près. La fontaine redevient une fontaine, tout simple.</t>
         </is>
       </c>
       <c r="F75" s="2" t="inlineStr">
         <is>
-          <t>Loin de l'eau, le rouge était là. Tu as fini, papa. Oui, le mot était long. Merci d'avoir reculé sans crier. La bourse cliquette une fois, puis se tait. Une goutte sèche déjà sur le bâton. Victorino fait tourner le rouge, tout près. La fontaine redevient une fontaine, tout simple.</t>
+          <t>Loin de l'eau, le rouge était là. Tu as fini, papa. Oui, le mot était long. Tu as reculé, tout doux. La bourse cliquette une fois, puis se tait. Une goutte sèche déjà sur le bâton. Victorino fait tourner le rouge, tout près. La fontaine redevient une fontaine, tout simple.</t>
         </is>
       </c>
       <c r="G75" s="2" t="inlineStr">
@@ -14402,7 +14402,7 @@
           <t>narrateur|Loin de l'eau, le rouge était là.
 enfant-m|Tu as fini, papa.
 papa|Oui, le mot était long.
-maman|Merci d'avoir reculé sans crier.
+maman|Tu as reculé, tout doux.
 narrateur|La bourse cliquette une fois, puis se tait.
 narrateur|Une goutte sèche déjà sur le bâton.
 narrateur|Victorino fait tourner le rouge, tout près.
@@ -15131,12 +15131,12 @@
       </c>
       <c r="E80" s="2" t="inlineStr">
         <is>
-          <t>La bourse arrive sous l'auvent bleu. La bourse n'atteint pas le bord, trop haute. Tout en haut ? Tout en haut, près du. Papa s'arrête, les lèvres encore rondes. Près du bord ? Victorino garde sa bouche fermée, après. Le haut est trop loin, pour lui. Un tabouret dort près du mur. Tu fais quoi, alors ?</t>
+          <t>La bourse arrive sous l'auvent bleu. Elle n'atteint pas le bord, trop haute. Tout en haut ? Tout en haut, près du. Papa s'arrête, les lèvres encore rondes. Près du bord ? Victorino garde sa bouche fermée, après. Le haut est trop loin, pour lui. Un tabouret dort près du mur. Tu fais quoi, alors ?</t>
         </is>
       </c>
       <c r="F80" s="2" t="inlineStr">
         <is>
-          <t>La bourse arrive sous l'auvent bleu. La bourse n'atteint pas le bord, trop haute. Tout en haut ? Tout en haut, près du. Papa s'arrête, les lèvres encore rondes. Près du bord ? Victorino garde sa bouche fermée, après. Le haut est trop loin, pour lui. Un tabouret dort près du mur. Tu fais quoi, alors ?</t>
+          <t>La bourse arrive sous l'auvent bleu. Elle n'atteint pas le bord, trop haute. Tout en haut ? Tout en haut, près du. Papa s'arrête, les lèvres encore rondes. Près du bord ? Victorino garde sa bouche fermée, après. Le haut est trop loin, pour lui. Un tabouret dort près du mur. Tu fais quoi, alors ?</t>
         </is>
       </c>
       <c r="G80" s="2" t="inlineStr">
@@ -15272,7 +15272,7 @@
       <c r="AW80" t="inlineStr">
         <is>
           <t>narrateur|La bourse arrive sous l'auvent bleu.
-narrateur|La bourse n'atteint pas le bord, trop haute.
+narrateur|Elle n'atteint pas le bord, trop haute.
 enfant-m|Tout en haut ?
 papa|Tout en haut, près du.
 narrateur|Papa s'arrête, les lèvres encore rondes.
@@ -16544,7 +16544,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A14"/>
+  <dimension ref="A1:A15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="100" customWidth="1" min="1" max="1"/>
@@ -16643,6 +16643,13 @@
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
+        <is>
+          <t>F-NAR-008 récit, pas une leçon en puces</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
         <is>
           <t>F-NAR-008 récit, pas une leçon en puces</t>
         </is>

</xml_diff>